<commit_message>
Add consequences to key Powell and Mead elevations data file
</commit_message>
<xml_diff>
--- a/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
+++ b/AutoReadUSBRData/ReservoirElevationDefinitions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Rosenberg\Work\USU\Research\ColoradoRiver\RCode\ColoradoRiverCollaborate\AutoReadUSBRData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A4741D9-F0FF-4F19-AC5F-4E935F837BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93E988A9-6564-4F69-98E8-ABFBF40E39BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
+    <workbookView xWindow="-28920" yWindow="-1965" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{8459C475-5003-475B-AAB9-94E9EA45958F}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="2" r:id="rId1"/>
@@ -22,14 +22,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="37">
   <si>
     <t>Reservoir</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>Mead</t>
   </si>
   <si>
@@ -109,6 +106,33 @@
   </si>
   <si>
     <t>No Hydropower (Vortices)</t>
+  </si>
+  <si>
+    <t>No hydropower generation or delivery to 9 western U.S. states</t>
+  </si>
+  <si>
+    <t>Vortices in penstocks</t>
+  </si>
+  <si>
+    <t>Risk</t>
+  </si>
+  <si>
+    <t>No downstream delivery to Lower Basin states and Mexico</t>
+  </si>
+  <si>
+    <t>No downstream delivery to CA, AZ, NV, and Mexico</t>
+  </si>
+  <si>
+    <t>No hydropower generation and delivery to Los Angeles, Las Vegas, or Phoenix</t>
+  </si>
+  <si>
+    <t>Invasive fish pass though dam, spread, and threaten native fish</t>
+  </si>
+  <si>
+    <t>Consequence</t>
+  </si>
+  <si>
+    <t>Invasive fish move into Grand Canyon and threaten native fish</t>
   </si>
 </sst>
 </file>
@@ -978,31 +1002,31 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1012,7 +1036,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8FD67FD-F240-49E2-BF91-7D417E153654}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="16.90625" customWidth="1"/>
@@ -1023,43 +1047,49 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
       </c>
       <c r="C2">
         <v>895</v>
       </c>
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3">
-        <v>955</v>
+        <v>950</v>
+      </c>
+      <c r="D3" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4">
         <v>975</v>
@@ -1067,10 +1097,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5">
         <v>1000</v>
@@ -1078,10 +1108,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6">
         <v>1020</v>
@@ -1089,10 +1119,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C7">
         <v>1025</v>
@@ -1100,10 +1130,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C8">
         <v>1050</v>
@@ -1111,10 +1141,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C9">
         <v>1090</v>
@@ -1122,24 +1152,44 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C10">
         <v>1135</v>
       </c>
+      <c r="D10" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11">
         <v>1218</v>
+      </c>
+      <c r="D11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>1</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12">
+        <v>1220</v>
+      </c>
+      <c r="D12" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1161,43 +1211,49 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
         <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
       </c>
       <c r="C2">
         <v>3370</v>
       </c>
+      <c r="D2" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C3">
         <v>3490</v>
       </c>
+      <c r="D3" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4">
         <v>3500</v>
@@ -1205,32 +1261,38 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C5">
         <v>3514</v>
       </c>
+      <c r="D5" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C6">
         <v>3525</v>
       </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7">
         <v>3535</v>
@@ -1238,10 +1300,10 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8">
         <v>3575</v>
@@ -1249,10 +1311,10 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9">
         <v>3600</v>
@@ -1260,13 +1322,16 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10">
         <v>3700</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>